<commit_message>
Study log May 18 2026 — DE+DS — 6.0hrs — 0 SQL
</commit_message>
<xml_diff>
--- a/Study_Progress_Tracker.xlsx
+++ b/Study_Progress_Tracker.xlsx
@@ -1145,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L253"/>
+  <dimension ref="A1:M253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1236,17 +1236,58 @@
       <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="10" t="inlineStr"/>
-      <c r="D4" s="10" t="inlineStr"/>
-      <c r="E4" s="9" t="inlineStr"/>
-      <c r="F4" s="10" t="inlineStr"/>
-      <c r="G4" s="10" t="inlineStr"/>
-      <c r="H4" s="10" t="inlineStr"/>
-      <c r="I4" s="10" t="inlineStr"/>
-      <c r="J4" s="10" t="inlineStr"/>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>May 18 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>May — Month 1</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>DE+DS</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Pandas Groupby Merge</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>Basic And Complex Datatypes Including Collection Module (Defaultdict</t>
+        </is>
+      </c>
       <c r="K4" s="9" t="inlineStr"/>
-      <c r="L4" s="9" t="inlineStr"/>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Normalization Concepts And Defaultdict Needs Revision   Insight: Merge In Pandas = Join In Sql</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Merge In Pandas = Join In Sql</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="7" t="n">

</xml_diff>